<commit_message>
Ajustarndo errores y validaciones
</commit_message>
<xml_diff>
--- a/public/plantillas/09_FUERZA_TRABAJO.xlsx
+++ b/public/plantillas/09_FUERZA_TRABAJO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B4C237-B568-B64F-8959-7D735B730584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802705B0-174D-174F-8868-EFD019892E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -102,6 +102,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -304,20 +307,20 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -675,7 +678,7 @@
     <row r="3" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="22"/>
+      <c r="D3" s="18"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="12"/>
@@ -721,8 +724,8 @@
       <c r="C5" s="16"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
       <c r="H5" s="15"/>
       <c r="I5" s="14"/>
       <c r="J5" s="17"/>

</xml_diff>

<commit_message>
Ajustando archivo de Fuerza de Trabajo
</commit_message>
<xml_diff>
--- a/public/plantillas/09_FUERZA_TRABAJO.xlsx
+++ b/public/plantillas/09_FUERZA_TRABAJO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802705B0-174D-174F-8868-EFD019892E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DF34F7-1B5D-8D48-94D4-C6DECE7ED824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -103,7 +103,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -310,6 +310,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -317,9 +320,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -413,44 +413,49 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>10440</xdr:colOff>
+      <xdr:colOff>38778</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>1800</xdr:rowOff>
+      <xdr:rowOff>48471</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>707760</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>145380</xdr:rowOff>
+      <xdr:colOff>998550</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>229980</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AE7B3577-8A8B-7FB7-6E23-F0164F98D579}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect l="3817" t="46435" r="77063" b="28961"/>
-        <a:stretch/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10440" y="1800"/>
-          <a:ext cx="1573620" cy="295980"/>
+          <a:off x="38778" y="48471"/>
+          <a:ext cx="1832291" cy="530517"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -661,19 +666,19 @@
       <c r="J1" s="7"/>
     </row>
     <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="19" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="19"/>
+      <c r="J2" s="20"/>
     </row>
     <row r="3" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="13"/>
@@ -683,8 +688,8 @@
       <c r="F3" s="13"/>
       <c r="G3" s="12"/>
       <c r="H3" s="8"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
     </row>
     <row r="4" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
@@ -724,8 +729,8 @@
       <c r="C5" s="16"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
       <c r="H5" s="15"/>
       <c r="I5" s="14"/>
       <c r="J5" s="17"/>

</xml_diff>

<commit_message>
Ajustando plantilla para exportar FT
</commit_message>
<xml_diff>
--- a/public/plantillas/09_FUERZA_TRABAJO.xlsx
+++ b/public/plantillas/09_FUERZA_TRABAJO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DF34F7-1B5D-8D48-94D4-C6DECE7ED824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B445F64-719C-6145-922D-17F0F7232E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -105,7 +105,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -186,6 +186,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -254,7 +261,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -320,6 +327,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -732,7 +742,7 @@
       <c r="F5" s="19"/>
       <c r="G5" s="19"/>
       <c r="H5" s="15"/>
-      <c r="I5" s="14"/>
+      <c r="I5" s="23"/>
       <c r="J5" s="17"/>
     </row>
     <row r="1048035" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Ajustando landing con funcionalidades especificas de diseño
</commit_message>
<xml_diff>
--- a/public/plantillas/09_FUERZA_TRABAJO.xlsx
+++ b/public/plantillas/09_FUERZA_TRABAJO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B445F64-719C-6145-922D-17F0F7232E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D21335F-0D29-F64F-B2DB-0B7181CCCC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Hoja 1'!$A$1:$J$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Hoja 1'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -320,6 +319,9 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -327,9 +329,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -652,14 +651,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:XFA1048076"/>
+  <dimension ref="A1:XFA1048074"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" style="1"/>
     <col min="2" max="2" width="38.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" style="2" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="31.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="33.83203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.83203125" style="4" customWidth="1"/>
     <col min="7" max="7" width="11.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" style="5" customWidth="1"/>
@@ -676,19 +675,19 @@
       <c r="J1" s="7"/>
     </row>
     <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="20" t="s">
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="20"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="3" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="13"/>
@@ -698,8 +697,8 @@
       <c r="F3" s="13"/>
       <c r="G3" s="12"/>
       <c r="H3" s="8"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
     </row>
     <row r="4" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
@@ -742,9 +741,11 @@
       <c r="F5" s="19"/>
       <c r="G5" s="19"/>
       <c r="H5" s="15"/>
-      <c r="I5" s="23"/>
+      <c r="I5" s="20"/>
       <c r="J5" s="17"/>
     </row>
+    <row r="1048033" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1048034" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1048035" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1048036" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1048037" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -785,8 +786,6 @@
     <row r="1048072" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1048073" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1048074" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048075" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048076" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="I2:J3"/>
@@ -794,7 +793,7 @@
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="69" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="67" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se crea modo demo
</commit_message>
<xml_diff>
--- a/public/plantillas/09_FUERZA_TRABAJO.xlsx
+++ b/public/plantillas/09_FUERZA_TRABAJO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventura/Desktop/Programacion/recal-hse/public/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D21335F-0D29-F64F-B2DB-0B7181CCCC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE35BF5-1BBD-D540-AF2D-B42D945CC457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3620" yWindow="0" windowWidth="29980" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -91,10 +91,10 @@
     <t>PERSONAL FORANEO</t>
   </si>
   <si>
-    <t>PROYECTO: PROYECTO: "REHABILITACION, SUSTITUCION Y/O MODERNIZACION DE 526 PUENTES DE LA LINEA K"</t>
-  </si>
-  <si>
     <t>NOMBRE DEL TRABAJADOR                (APELLIDOS-NOMBRES)</t>
+  </si>
+  <si>
+    <t>PROYECTO: "REHABILITACION, SUSTITUCION Y/O MODERNIZACION DE 526 PUENTES DE LA LINEA K"</t>
   </si>
 </sst>
 </file>
@@ -676,7 +676,7 @@
     </row>
     <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="22"/>
       <c r="D2" s="22"/>
@@ -705,7 +705,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>3</v>

</xml_diff>